<commit_message>
Daily facility note collection 2026-09-06
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1428,6 +1428,996 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>しぶそば自由が丘店</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.shibusoba.com/post/jyugaokaopen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>近江ちゃんぽん亭 岩出店</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://dreamfoods.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>&lt;10/27予定&gt;スーパーマーケットバロー大府北山店</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>10/29 オーケー長吉店(大阪市)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eUx</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>&lt;11/28予定&gt;ドラッグコスモス印場橋店(愛知県)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1e1s</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>&lt;1/29予定&gt; ザ・ビッグエクストラ関店(岐阜県関市)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eOu</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>業務スーパー秋田保戸野店2026年7月30日オープン,【1.9万表示】2026/07/</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://x.com/shokusaijp_TMGP/status/2081561660947677395</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026年09月06日</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily facility note collection 2026-09-07
</commit_message>
<xml_diff>
--- a/data/store_openings.xlsx
+++ b/data/store_openings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2418,6 +2418,1326 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>9/10とりせん田沼インター店(栃木県佐野市)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>暮らしと不動産の窓口 K-LIVING ESTATE</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://kl-estate.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>おたからや 上野マルイ店</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.otakaraya.jp/shop/ueno-m/</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>アトリエうかい Cafe &amp; Factory HACHIOJI</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.ukai.co.jp/atelier/cafe-factory/</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>焼肉 塩ホルモン 好ちゃん 神田本店</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://selecao.co.jp/ourshops/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>エリックサウス</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://enso.ne.jp/erick-south/</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>和食日和 おさけと 大手町</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.osaketo-washoku.jp/shop/otemachi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ブラッスリー・ローデンバッハ</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.rodenbach.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>ドトールコーヒーショップ 大手町ゲートビルディング店</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.doutor.co.jp/dcs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>大衆とり酒場 とりいちず 大森東口店</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://toriichizu.net/shoplist/4044/</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>壱角家 八重洲店</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://gardengroup.co.jp/brand/ichikakuya/</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>IL BISONTE 玉川高島屋S・C店</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.ilbisonte.jp/shops/kanto?c=tamagawa_takashimaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Meet＆Meat produced by 相席屋</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://section-8.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>スターバックス コーヒー 長野若槻店</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://store.starbucks.co.jp/detail-4623/</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>かにじぇんぬ 金沢</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kani.kanazawa/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>VIENT（ビエント）近江八幡店</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://vient-pilates.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>牛角焼肉食堂＆ホルモン酒場 阪神梅田本店スナックパーク店</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.reins.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>近江ちゃんぽん亭 岩出店</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://chanpontei.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ワッツウィズ河南町キリン堂店</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.watts-jp.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>10/9TAKENOKO＋byFOODSMARKETsatakeビエラ千里丘</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g98</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>百十四銀行 坂出支店</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.114bank.co.jp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>牛角焼肉食堂 ゆめタウン久留米店</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://gyukakuyakinikushokudou.ne.jp/store/detail/?id=yumetownkurume</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>9/1オーケー高槻赤大路店(大阪府高槻市)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fOy</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>9/1 ライフ鎌倉梶原店</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fS5</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>9/3 サンディ吹田五月が丘店(大阪府吹田市)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fPd</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>9/3改装 スーパーのアオキ直江津店(新潟県上越市)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2v</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>9/3スギ薬局茜部南店(岐阜市)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g2N</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>9/4クックマート上西店（静岡県浜松市）</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7N</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>9/4(9/3プレ)スーパー生鮮館TAIGA桂子田店</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fZU</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>9/4改装 名古屋PARCO</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7c</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>9/4改装 メイチカ(名古屋市)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7g</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>9/4ウルフギャングステーキハウス名古屋店</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1eZr</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>9/4 ゴジラ・ストア Nagoya</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fn6</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>9/4ロピア彦根ナフコ店</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>9/10改装 マルナカ檀紙店(香川県高松市)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g7X</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>9/10ザ・ビッグエクスプレスみよし店</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>9/10ファミリーマート中津川下野店</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g84</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>9/11スーパーマーケットバロー豊中島江店</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fXN</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>9/16SANYO Style STORE PLUS イオンモール岡崎店</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1fEw</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>食彩品館NEWS</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>9/17ロピア ムサシ新潟西店(新潟市)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://wp.me/pg0IT6-1g6X</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>9月1日(火)OPEN！「KINUJO」の世界観を五感で楽しむ『KINUJO Cafe &amp; Bar』が銀座の地に誕生。洗練されたインテリアと美食が融合した特別な体験をお届けいたします。</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000048.000094687.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>【2026年9月3日(木)オープン】全国の名品・銘菓を集めた新店舗「日本めぐり はくまる庵」が誕生</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000003.000188020.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>A5黒毛和牛をひつまぶしスタイルで味わう新ランチが誕生。「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」にて、7月20日（月）より『A5黒毛和牛の博多牛まぶし』の提供を開始</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000019.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>【大阪・天王寺に山椒まぜそば登場】痺れと香りを極めた山椒まぜそば専門店『麺処 山椒』が2026年7月25日（土）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000015.000055652.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>新潟市内、フレスポ赤道に登場！ナポリタン専門店「スパゲッティーのパンチョ 新潟赤道店」が7月17日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000105.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>新潟市南区に「あくあしょっぷ　ぎんなん」7月7日OPEN｜海水魚・水草・生体を扱う、小さく始められるアクアリウム専門店</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000002.000186660.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>【オープン記念としておすすめコースに飲み放題を無料提供】香りを愉しむ新業態「薪焼きともつ鍋 桂香-KEIKA- 博多西中洲」が7月6日（月）グランドオープン！7月1日（水）よりプレオープン</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000018.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>栃木初上陸、全国50店舗目の節目を飾る！ナポリタン専門店「スパゲッティーのパンチョ 宇都宮戸祭店」が7月3日（金）に新規開店、3連続オープニングキャンペーンを開催</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000103.000117096.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>【生ビール・角ハイボール・鬼おろしレモンサワー78円】旬を摘まむオトナ酒場「酒と肴 菜の華(なのはな) 銀座通り店」が6月1日(月)グランドオープン！6月30日(火)まで一部ドリンクを破格でご提供！</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000017.000106843.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026年09月07日</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>PR TIMES</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>【和食さと】広島県に初出店！「和食さと広島観音新町店」を2026年5月22日（金）グランドオープン！</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>/main/html/rd/p/000000899.000122416.html</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>